<commit_message>
environment dsa updated upto 2025
</commit_message>
<xml_diff>
--- a/Environment/Original Data/environment reference sheet.xlsx
+++ b/Environment/Original Data/environment reference sheet.xlsx
@@ -62,7 +62,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -84,11 +84,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -105,6 +149,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -591,23 +637,23 @@
           <t>-- Water --</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
+      <c r="B2" s="6" t="n"/>
+      <c r="C2" s="6" t="n"/>
+      <c r="D2" s="6" t="n"/>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="n"/>
+      <c r="M2" s="6" t="n"/>
+      <c r="N2" s="6" t="n"/>
+      <c r="O2" s="6" t="n"/>
+      <c r="P2" s="6" t="n"/>
+      <c r="Q2" s="6" t="n"/>
+      <c r="R2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -1605,23 +1651,23 @@
           <t>-- Climate &amp; Atmosphere --</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
-      <c r="M14" s="3" t="n"/>
-      <c r="N14" s="3" t="n"/>
-      <c r="O14" s="3" t="n"/>
-      <c r="P14" s="3" t="n"/>
-      <c r="Q14" s="3" t="n"/>
-      <c r="R14" s="3" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="6" t="n"/>
+      <c r="M14" s="6" t="n"/>
+      <c r="N14" s="6" t="n"/>
+      <c r="O14" s="6" t="n"/>
+      <c r="P14" s="6" t="n"/>
+      <c r="Q14" s="6" t="n"/>
+      <c r="R14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -2259,23 +2305,23 @@
           <t>-- Forests &amp; Ecology --</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
-      <c r="L22" s="3" t="n"/>
-      <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3" t="n"/>
-      <c r="O22" s="3" t="n"/>
-      <c r="P22" s="3" t="n"/>
-      <c r="Q22" s="3" t="n"/>
-      <c r="R22" s="3" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
+      <c r="J22" s="6" t="n"/>
+      <c r="K22" s="6" t="n"/>
+      <c r="L22" s="6" t="n"/>
+      <c r="M22" s="6" t="n"/>
+      <c r="N22" s="6" t="n"/>
+      <c r="O22" s="6" t="n"/>
+      <c r="P22" s="6" t="n"/>
+      <c r="Q22" s="6" t="n"/>
+      <c r="R22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -2553,23 +2599,23 @@
           <t>-- Human Footprint --</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n"/>
-      <c r="I26" s="3" t="n"/>
-      <c r="J26" s="3" t="n"/>
-      <c r="K26" s="3" t="n"/>
-      <c r="L26" s="3" t="n"/>
-      <c r="M26" s="3" t="n"/>
-      <c r="N26" s="3" t="n"/>
-      <c r="O26" s="3" t="n"/>
-      <c r="P26" s="3" t="n"/>
-      <c r="Q26" s="3" t="n"/>
-      <c r="R26" s="3" t="n"/>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
+      <c r="I26" s="6" t="n"/>
+      <c r="J26" s="6" t="n"/>
+      <c r="K26" s="6" t="n"/>
+      <c r="L26" s="6" t="n"/>
+      <c r="M26" s="6" t="n"/>
+      <c r="N26" s="6" t="n"/>
+      <c r="O26" s="6" t="n"/>
+      <c r="P26" s="6" t="n"/>
+      <c r="Q26" s="6" t="n"/>
+      <c r="R26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -18585,11 +18631,11 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>502</v>
+        <v>752</v>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>2009-2021</t>
+          <t>2009-2024</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -18616,11 +18662,11 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>4352</v>
+        <v>6016</v>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>2006-2021</t>
+          <t>2006-2024</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -18647,11 +18693,11 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>1076</v>
+        <v>1492</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>2009-2021</t>
+          <t>2009-2024</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -18740,11 +18786,11 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>2770</v>
+        <v>3832</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>2006-2021</t>
+          <t>2006-2024</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">

</xml_diff>